<commit_message>
feat: implement interactive image zooming and lightbox for poll options, and add dedicated voting results pages.
</commit_message>
<xml_diff>
--- a/Membership_Reg_(Course)_(Year)_(Section).xlsx
+++ b/Membership_Reg_(Course)_(Year)_(Section).xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robprisoris/Documents/GithubProjects/OrgWeb/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783E590C-0DE1-4F48-AEB2-7717CA7C0183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="2100" yWindow="600" windowWidth="34200" windowHeight="19500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1 - members_sample" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet 1 - members_sample" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
-  <si>
-    <t>members_sample</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Student ID</t>
   </si>
@@ -40,65 +46,33 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Membership Status</t>
-  </si>
-  <si>
-    <t>Payment</t>
-  </si>
-  <si>
-    <t>2024-0001</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
-    <t>Doe</t>
-  </si>
-  <si>
     <t>BSIT</t>
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>BSCE</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
   <si>
     <r>
       <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>john.doe@example.com</t>
-    </r>
-  </si>
-  <si>
-    <t>Half Semester Paid</t>
-  </si>
-  <si>
-    <t>2024-0002</t>
-  </si>
-  <si>
-    <t>Jane</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>BSCE</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
+        <u/>
         <sz val="10"/>
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
@@ -107,12 +81,6 @@
     </r>
   </si>
   <si>
-    <t>Partial</t>
-  </si>
-  <si>
-    <t>2024-0003</t>
-  </si>
-  <si>
     <t>Alice</t>
   </si>
   <si>
@@ -130,7 +98,7 @@
   <si>
     <r>
       <rPr>
-        <u val="single"/>
+        <u/>
         <sz val="10"/>
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
@@ -139,12 +107,6 @@
     </r>
   </si>
   <si>
-    <t>Not Paid</t>
-  </si>
-  <si>
-    <t>2024-0004</t>
-  </si>
-  <si>
     <t>Bob</t>
   </si>
   <si>
@@ -159,7 +121,7 @@
   <si>
     <r>
       <rPr>
-        <u val="single"/>
+        <u/>
         <sz val="10"/>
         <color indexed="8"/>
         <rFont val="Helvetica Neue"/>
@@ -167,36 +129,66 @@
       <t>bob.brown@company.com</t>
     </r>
   </si>
+  <si>
+    <t>2024-0022</t>
+  </si>
+  <si>
+    <t>2024-0026</t>
+  </si>
+  <si>
+    <t>2024-0023</t>
+  </si>
+  <si>
+    <t>2024-0025</t>
+  </si>
+  <si>
+    <t>Mark</t>
+  </si>
+  <si>
+    <t>maek</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -334,45 +326,48 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -383,26 +378,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="ffdbdbdb"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFBDC0BF"/>
+      <rgbColor rgb="FFA5A5A5"/>
+      <rgbColor rgb="FF3F3F3F"/>
+      <rgbColor rgb="FFDBDBDB"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Blank">
   <a:themeElements>
     <a:clrScheme name="Blank">
       <a:dk1>
@@ -601,7 +655,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -619,7 +673,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1200" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -648,7 +702,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -673,7 +727,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -698,7 +752,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -723,7 +777,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -748,7 +802,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -773,7 +827,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -798,7 +852,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -823,7 +877,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -848,7 +902,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -861,9 +915,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -880,7 +940,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -898,7 +958,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -923,7 +983,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -948,7 +1008,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -973,7 +1033,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -998,7 +1058,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1023,7 +1083,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1048,7 +1108,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1073,7 +1133,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1098,7 +1158,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1123,7 +1183,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1136,9 +1196,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1152,7 +1218,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1170,7 +1236,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1199,7 +1265,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1224,7 +1290,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1249,7 +1315,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1274,7 +1340,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1299,7 +1365,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1324,7 +1390,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1349,7 +1415,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1374,7 +1440,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1399,7 +1465,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1412,231 +1478,187 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:J6"/>
-  <sheetFormatPr defaultColWidth="8.33333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.85156" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1719" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.17188" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.1640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="21.3516" style="1" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="17" style="1" customWidth="1"/>
     <col min="10" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.35156" style="1" customWidth="1"/>
+    <col min="11" max="11" width="8.33203125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" t="s" s="3">
+    <row r="2" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="4">
+        <v>3</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="7">
+        <v>2</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="7">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="3">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s" s="3">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s" s="3">
+      <c r="H4" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="7">
         <v>4</v>
       </c>
-      <c r="E2" t="s" s="3">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s" s="3">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s" s="3">
-        <v>7</v>
-      </c>
-      <c r="H2" t="s" s="3">
-        <v>8</v>
-      </c>
-      <c r="I2" t="s" s="3">
-        <v>9</v>
-      </c>
-      <c r="J2" t="s" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" t="s" s="4">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s" s="5">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s" s="6">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s" s="6">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s" s="6">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s" s="6">
-        <v>16</v>
-      </c>
-      <c r="G3" s="7">
-        <v>3</v>
-      </c>
-      <c r="H3" t="s" s="6">
-        <v>17</v>
-      </c>
-      <c r="I3" t="s" s="6">
-        <v>18</v>
-      </c>
-      <c r="J3" s="7">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" t="s" s="8">
-        <v>19</v>
-      </c>
-      <c r="B4" t="s" s="9">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s" s="10">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="E4" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>24</v>
-      </c>
-      <c r="G4" s="11">
-        <v>2</v>
-      </c>
-      <c r="H4" t="s" s="10">
-        <v>25</v>
-      </c>
-      <c r="I4" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="J4" s="11">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" t="s" s="8">
+      <c r="H5" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" t="s" s="9">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s" s="10">
-        <v>30</v>
-      </c>
-      <c r="E5" t="s" s="10">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G5" s="11">
-        <v>1</v>
-      </c>
-      <c r="H5" t="s" s="10">
-        <v>33</v>
-      </c>
-      <c r="I5" t="s" s="10">
-        <v>34</v>
-      </c>
-      <c r="J5" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" t="s" s="8">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s" s="9">
-        <v>36</v>
-      </c>
-      <c r="C6" t="s" s="10">
-        <v>37</v>
-      </c>
-      <c r="D6" t="s" s="10">
-        <v>38</v>
-      </c>
-      <c r="E6" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="F6" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="G6" s="11">
-        <v>4</v>
-      </c>
-      <c r="H6" t="s" s="10">
-        <v>40</v>
-      </c>
-      <c r="I6" t="s" s="10">
-        <v>18</v>
-      </c>
-      <c r="J6" s="11">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E6">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"BSIT,BSCE,BITM,BSM,BSMRS"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I6">
-      <formula1>"Fully Paid,Partial,Not Paid,Half Semester Paid"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" location="" tooltip="" display="john.doe@example.com"/>
-    <hyperlink ref="H4" r:id="rId2" location="" tooltip="" display="jane.smith@example.org"/>
-    <hyperlink ref="H5" r:id="rId3" location="" tooltip="" display="alice.j@uni.edu"/>
-    <hyperlink ref="H6" r:id="rId4" location="" tooltip="" display="bob.brown@company.com"/>
+    <hyperlink ref="H3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="H5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H2" r:id="rId4" display="john.doe@example.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
feat: implement role-based access control for attendance scanners and treasurers with updated navigation and login routing
</commit_message>
<xml_diff>
--- a/Membership_Reg_(Course)_(Year)_(Section).xlsx
+++ b/Membership_Reg_(Course)_(Year)_(Section).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robprisoris/Documents/GithubProjects/OrgWeb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783E590C-0DE1-4F48-AEB2-7717CA7C0183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB43642A-0FBB-B345-91DB-6453C4E64112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="600" windowWidth="34200" windowHeight="19500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2100" yWindow="600" windowWidth="34200" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - members_sample" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Student ID</t>
   </si>
@@ -53,18 +53,6 @@
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>Jane</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>BSCE</t>
   </si>
   <si>
     <t>B</t>
@@ -81,71 +69,31 @@
     </r>
   </si>
   <si>
-    <t>Alice</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Johnson</t>
-  </si>
-  <si>
     <t>BITM</t>
   </si>
   <si>
     <t>C</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>alice.j@uni.edu</t>
-    </r>
-  </si>
-  <si>
-    <t>Bob</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>BSM</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>bob.brown@company.com</t>
-    </r>
-  </si>
-  <si>
-    <t>2024-0022</t>
-  </si>
-  <si>
-    <t>2024-0026</t>
-  </si>
-  <si>
     <t>2024-0023</t>
   </si>
   <si>
-    <t>2024-0025</t>
-  </si>
-  <si>
-    <t>Mark</t>
-  </si>
-  <si>
-    <t>maek</t>
+    <t>Kirt</t>
+  </si>
+  <si>
+    <t>Basog</t>
+  </si>
+  <si>
+    <t>kirt@gmail.com</t>
+  </si>
+  <si>
+    <t>0001-0001</t>
+  </si>
+  <si>
+    <t>Joomer Jake</t>
+  </si>
+  <si>
+    <t>Caballero</t>
   </si>
 </sst>
 </file>
@@ -186,9 +134,8 @@
     <font>
       <u/>
       <sz val="10"/>
-      <color indexed="8"/>
+      <color theme="10"/>
       <name val="Helvetica Neue"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -325,12 +272,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -344,9 +294,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -367,11 +314,18 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1500,7 +1454,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.83203125" style="1" customWidth="1"/>
@@ -1544,15 +1498,17 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="8"/>
+      <c r="A2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>16</v>
+      </c>
       <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="11" t="s">
-        <v>32</v>
+      <c r="D2" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>9</v>
@@ -1563,99 +1519,45 @@
       <c r="G2" s="4">
         <v>3</v>
       </c>
-      <c r="H2" s="12" t="s">
-        <v>33</v>
+      <c r="H2" s="11" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="G3" s="6">
+        <v>3</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="7">
-        <v>2</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="7">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="7">
-        <v>4</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"BSIT,BSCE,BITM,BSM,BSMRS"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="H4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="H5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="H2" r:id="rId4" display="john.doe@example.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
feat: refactor hero section with real-time stats and branding updates
</commit_message>
<xml_diff>
--- a/Membership_Reg_(Course)_(Year)_(Section).xlsx
+++ b/Membership_Reg_(Course)_(Year)_(Section).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robprisoris/Documents/GithubProjects/OrgWeb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Rob Buids/Website Projects/OrgWeb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB43642A-0FBB-B345-91DB-6453C4E64112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873E5337-51B8-344F-BE0D-7A5EBE4A6AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="600" windowWidth="34200" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14960" yWindow="3280" windowWidth="34200" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - members_sample" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Student ID</t>
   </si>
@@ -46,74 +46,33 @@
     <t>Email</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
     <t>BSIT</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>jane.smith@example.org</t>
-    </r>
-  </si>
-  <si>
-    <t>BITM</t>
   </si>
   <si>
     <t>C</t>
   </si>
   <si>
-    <t>2024-0023</t>
+    <t>M</t>
   </si>
   <si>
-    <t>Kirt</t>
+    <t>roberto.prisoris12@gmail.com</t>
   </si>
   <si>
-    <t>Basog</t>
+    <t>2022-2703</t>
   </si>
   <si>
-    <t>kirt@gmail.com</t>
+    <t>Roberto Jr</t>
   </si>
   <si>
-    <t>0001-0001</t>
-  </si>
-  <si>
-    <t>Joomer Jake</t>
-  </si>
-  <si>
-    <t>Caballero</t>
+    <t>Prisoris</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <u/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -136,6 +95,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -158,7 +118,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -226,61 +186,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -296,31 +211,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1464,7 +1364,7 @@
     <col min="5" max="5" width="7.1640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" style="1" customWidth="1"/>
     <col min="10" max="10" width="8.5" style="1" customWidth="1"/>
     <col min="11" max="11" width="8.33203125" style="1" customWidth="1"/>
@@ -1499,65 +1399,39 @@
     </row>
     <row r="2" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="4">
-        <v>3</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>18</v>
+        <v>4</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="6">
-        <v>3</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
+    <row r="3" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"BSIT,BSCE,BITM,BSM,BSMRS"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="H2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{52EAAFE2-123F-7449-AE57-F450EFE36269}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>